<commit_message>
Updated automation test file for T-P
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -473,20 +473,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The `frequency` column in the `campaign_performance` table represents the average number of times a user was exposed to an ad. It is a directly recorded metric within the table, not a derived field from other columns in this schema.</t>
+          <t>Error: 500 Server Error: Internal Server Error for url: http://127.0.0.1:8000/run</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.836</v>
+        <v>-0.018</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[{'invocationId': 'e-83203d58-7476-40f2-aa64-646157beb36e', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'yNynCm25', 'timestamp': 1757072566.122553}, {'content': {'parts': [{'text': 'The `frequency` column in the `campaign_performance` table represents the average number of times a user was exposed to an ad. It is a directly recorded metric within the table, not a derived field from other columns in this schema.'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 48, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 48}], 'promptTokenCount': 8238, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8238}], 'thoughtsTokenCount': 87, 'totalTokenCount': 8373, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-83203d58-7476-40f2-aa64-646157beb36e', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'Lq2HFlnm', 'timestamp': 1757072566.124085}]</t>
+          <t>Error: 500 Server Error: Internal Server Error for url: http://127.0.0.1:8000/run</t>
         </is>
       </c>
     </row>
@@ -508,16 +508,15 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The `transaction_data` and `campaign_performance` tables can be linked using the following fields:
-*   `campaign_id`
-*   `campaign_ad_id`
-*   `brand_id`
-*   `brand_name`
-*   `product_ids` (Note: `transaction_data` has `sku_id` which is a product identifier, and `campaign_performance` has `product_ids`. These are likely related and can be used for linking, but `campaign_id`, `campaign_ad_id`, `brand_id`, and `brand_name` are direct common fields.)</t>
+          <t>The fields that link `transaction_data` to `campaign_performance` are:
+- `campaign_id`
+- `campaign_ad_id`
+- `brand_id`
+- `brand_name`</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.806</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -526,7 +525,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[{'invocationId': 'e-53e9ea95-dcb7-49ea-9e32-cb36aa084b26', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': '76tvzSiR', 'timestamp': 1757072575.663537}, {'content': {'parts': [{'text': 'The `transaction_data` and `campaign_performance` tables can be linked using the following fields:\n\n*   `campaign_id`\n*   `campaign_ad_id`\n*   `brand_id`\n*   `brand_name`\n*   `product_ids` (Note: `transaction_data` has `sku_id` which is a product identifier, and `campaign_performance` has `product_ids`. These are likely related and can be used for linking, but `campaign_id`, `campaign_ad_id`, `brand_id`, and `brand_name` are direct common fields.)'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 135, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 135}], 'promptTokenCount': 8241, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8241}], 'thoughtsTokenCount': 359, 'totalTokenCount': 8735, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-53e9ea95-dcb7-49ea-9e32-cb36aa084b26', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'UyxqDIA6', 'timestamp': 1757072575.665663}]</t>
+          <t>[{'invocationId': 'e-d3de399b-5052-4c5a-8818-a313fbdc2057', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': '0D2M3vql', 'timestamp': 1757423714.88188}, {'content': {'parts': [{'text': 'The fields that link `transaction_data` to `campaign_performance` are:\n- `campaign_id`\n- `campaign_ad_id`\n- `brand_id`\n- `brand_name`'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 47, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 47}], 'promptTokenCount': 8268, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8268}], 'thoughtsTokenCount': 506, 'totalTokenCount': 8821, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-d3de399b-5052-4c5a-8818-a313fbdc2057', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'TdYZR2zw', 'timestamp': 1757423714.88302}]</t>
         </is>
       </c>
     </row>
@@ -544,43 +543,43 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CPC is a direct column in the `campaign_performance` table.</t>
+          <t>CPC is a pre-calculated metric available in the `campaign_performance` table.</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.733</v>
+        <v>0.837</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[{'invocationId': 'e-38fb7be2-f610-4fad-a483-2cfd54bb351c', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'xsODIdc6', 'timestamp': 1757072586.172655}, {'content': {'parts': [{'text': 'CPC is a direct column in the `campaign_performance` table.'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7609}], 'cachedContentTokenCount': 7609, 'candidatesTokenCount': 14, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 14}], 'promptTokenCount': 8237, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8237}], 'thoughtsTokenCount': 206, 'totalTokenCount': 8457, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-38fb7be2-f610-4fad-a483-2cfd54bb351c', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'kzpeQkDN', 'timestamp': 1757072586.175194}]</t>
+          <t>[{'invocationId': 'e-1ba751bb-ed3a-48fc-b9bb-4ed9e279bcc3', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': '2lCgQyWh', 'timestamp': 1757423723.956275}, {'content': {'parts': [{'text': 'CPC is a pre-calculated metric available in the `campaign_performance` table.'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 17, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 17}], 'promptTokenCount': 8264, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8264}], 'thoughtsTokenCount': 129, 'totalTokenCount': 8410, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-1ba751bb-ed3a-48fc-b9bb-4ed9e279bcc3', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': '0mgfBqZP', 'timestamp': 1757423723.95741}]</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>How is conversion_rate_percent defined in campaign_performance?</t>
+          <t>Show a bar chart of actual spend to date by channel.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The conversion_rate_percent in the campaign_performance table is a FLOAT type. It is typically calculated as:
-( conversions / clicks ) * 100
-This represents the percentage of clicks that resulted in a conversion.</t>
+          <t>Result: This bar chart effectively visualizes the actual spend to date across different channels. It clearly shows that 'Offsite' has the highest spend, followed by 'Onsite' and 'App', while 'Channel-CTV' and 'In-storeResult: This bar chart effectively visualizes the actual spend to date across different channels. It clearly shows that 'Offsite' has the highest spend, followed by 'Onsite' and 'App', while 'Channel-CTV' and 'In-store' represent significantly lower expenditures. This type of chart is useful for quickly identifying which channels are receiving the most investment.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>`conversion_rate_percent` in the `campaign_performance` table is defined as a `FLOAT`.</t>
+          <t xml:space="preserve">**Result:** The chart shows the actual spend to date by channel. Offsite channel has the highest spend, followed by Onsite and App channels. In-store channel has the lowest spend.
+Hope this was helpful! Let me know if you need to analyze other attributes or create more charts.
+</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.883</v>
+        <v>0.892</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -589,7 +588,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[{'invocationId': 'e-33020a5b-8ce4-4a63-af12-c09802a704a8', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'nYnykQcL', 'timestamp': 1757072596.815562}, {'content': {'parts': [{'text': '`conversion_rate_percent` in the `campaign_performance` table is defined as a `FLOAT`.'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 22, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 22}], 'promptTokenCount': 8242, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8242}], 'thoughtsTokenCount': 117, 'totalTokenCount': 8381, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-33020a5b-8ce4-4a63-af12-c09802a704a8', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'vrCwuBmT', 'timestamp': 1757072596.816599}]</t>
+          <t>[{'invocationId': 'e-ff1ff317-3386-47bc-a5ed-4660cd9b5551', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'JXCp4GRC', 'timestamp': 1757423730.98982}, {'content': {'parts': [{'functionCall': {'id': 'adk-ee36d06b-6458-487f-bc65-8f324ca9307d', 'args': {'question': 'What is the actual spend to date by channel?'}, 'name': 'call_db_agent'}}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 16, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 16}], 'promptTokenCount': 8268, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8268}], 'thoughtsTokenCount': 195, 'totalTokenCount': 8479, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-ff1ff317-3386-47bc-a5ed-4660cd9b5551', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'longRunningToolIds': [], 'id': 'Q3HmUHTj', 'timestamp': 1757423730.990813}, {'content': {'parts': [{'functionResponse': {'id': 'adk-ee36d06b-6458-487f-bc65-8f324ca9307d', 'name': 'call_db_agent', 'response': {'result': '```json\n{\n  "explain": "The SQL query calculates the sum of `actual_spend_to_date` for each `channels` from the `campaign_performance` table. It groups the results by `channels` to show the total spend for each channel.",\n  "sql": "SELECT\\n    t1.channels,\\n    SUM(t1.actual_spend_to_date) AS total_actual_spend_to_date\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n  GROUP BY\\n    t1.channels\\n  LIMIT 500",\n  "sql_results": [\n    {\n      "channels": "Onsite",\n      "total_actual_spend_to_date": 133455139.97500044\n    },\n    {\n      "channels": "App",\n      "total_actual_spend_to_date": 126214368.35499968\n    },\n    {\n      "channels": "Offsite",\n      "total_actual_spend_to_date": 156833302.079999\n    },\n    {\n      "channels": "Channel-CTV",\n      "total_actual_spend_to_date": 46984040.660000049\n    },\n    {\n      "channels": "In-store",\n      "total_actual_spend_to_date": 32660484.865000207\n    }\n  ],\n  "nl_results": "The actual spend to date by channel is:\\n- Onsite: 133,455,139.98\\n- App: 126,214,368.35\\n- Offsite: 156,833,302.08\\n- Channel-CTV: 46,984,040.66\\n- In-store: 32,660,484.87"\n}\n```'}}}], 'role': 'user'}, 'invocationId': 'e-ff1ff317-3386-47bc-a5ed-4660cd9b5551', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'sql_query': 'SELECT\n    t1.channels,\n    SUM(t1.actual_spend_to_date) AS total_actual_spend_to_date\n  FROM\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\n  GROUP BY\n    t1.channels\n  LIMIT 500', 'query_result': [{'channels': 'Onsite', 'total_actual_spend_to_date': 133455139.97500044}, {'channels': 'App', 'total_actual_spend_to_date': 126214368.35499968}, {'channels': 'Offsite', 'total_actual_spend_to_date': 156833302.079999}, {'channels': 'Channel-CTV', 'total_actual_spend_to_date': 46984040.66000005}, {'channels': 'In-store', 'total_actual_spend_to_date': 32660484.865000207}], 'db_agent_output': '```json\n{\n  "explain": "The SQL query calculates the sum of `actual_spend_to_date` for each `channels` from the `campaign_performance` table. It groups the results by `channels` to show the total spend for each channel.",\n  "sql": "SELECT\\n    t1.channels,\\n    SUM(t1.actual_spend_to_date) AS total_actual_spend_to_date\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n  GROUP BY\\n    t1.channels\\n  LIMIT 500",\n  "sql_results": [\n    {\n      "channels": "Onsite",\n      "total_actual_spend_to_date": 133455139.97500044\n    },\n    {\n      "channels": "App",\n      "total_actual_spend_to_date": 126214368.35499968\n    },\n    {\n      "channels": "Offsite",\n      "total_actual_spend_to_date": 156833302.079999\n    },\n    {\n      "channels": "Channel-CTV",\n      "total_actual_spend_to_date": 46984040.660000049\n    },\n    {\n      "channels": "In-store",\n      "total_actual_spend_to_date": 32660484.865000207\n    }\n  ],\n  "nl_results": "The actual spend to date by channel is:\\n- Onsite: 133,455,139.98\\n- App: 126,214,368.35\\n- Offsite: 156,833,302.08\\n- Channel-CTV: 46,984,040.66\\n- In-store: 32,660,484.87"\n}\n```'}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'g8U51ip1', 'timestamp': 1757423770.926473}, {'content': {'parts': [{'functionCall': {'id': 'adk-ffc5f37b-818c-4fd8-b29e-708f1807c504', 'args': {'question': 'Show a bar chart of actual spend to date by channel.'}, 'name': 'call_viz_agent'}}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7605}], 'cachedContentTokenCount': 7605, 'candidatesTokenCount': 18, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 18}], 'promptTokenCount': 8807, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8807}], 'thoughtsTokenCount': 126, 'totalTokenCount': 8951, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-ff1ff317-3386-47bc-a5ed-4660cd9b5551', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'longRunningToolIds': [], 'id': 'jsRvTtZ8', 'timestamp': 1757423770.929129}, {'content': {'parts': [{'functionResponse': {'id': 'adk-ffc5f37b-818c-4fd8-b29e-708f1807c504', 'name': 'call_viz_agent', 'response': {'text': 'The chart shows the actual spend to date by channel. Offsite channel has the highest spend, followed by Onsite and App channels. In-store channel has the lowest spend.\n\nHope this was helpful! Let me know if you need to analyze other attributes or create more charts.', 'images': []}}}], 'role': 'user'}, 'invocationId': 'e-ff1ff317-3386-47bc-a5ed-4660cd9b5551', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'chart_type': 'bar', 'x_axis_label': 'Channels', 'y_axis_label': 'Total Actual Spend To Date ($)', 'x': [], 'y': [], 'categories': ['Onsite', 'App', 'Offsite', 'Channel-CTV', 'In-store'], 'values': [133455139.97500044, 126214368.35499968, 156833302.079999, 46984040.66000005, 32660484.865000207], 'title': 'Actual Spend to Date by Channel', 'stages': [], 'subcategories': [], 'dv_agent_output': 'The chart shows the actual spend to date by channel. Offsite channel has the highest spend, followed by Onsite and App channels. In-store channel has the lowest spend.\n\nHope this was helpful! Let me know if you need to analyze other attributes or create more charts.'}, 'artifactDelta': {'chart_20250909_184630.png': 0}, 'requestedAuthConfigs': {}}, 'id': 'AAyLTKNS', 'timestamp': 1757423799.678888}, {'content': {'parts': [{'text': '**Result:** The chart shows the actual spend to date by channel. Offsite channel has the highest spend, followed by Onsite and App channels. In-store channel has the lowest spend.\n\nHope this was helpful! Let me know if you need to analyze other attributes or create more charts.\n'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7586}], 'cachedContentTokenCount': 7586, 'candidatesTokenCount': 61, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 61}], 'promptTokenCount': 8964, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8964}], 'thoughtsTokenCount': 114, 'totalTokenCount': 9139, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-ff1ff317-3386-47bc-a5ed-4660cd9b5551', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': '1RhCVeP7', 'timestamp': 1757423799.683231}]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
made changes in prompt and latency
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -473,20 +473,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The `frequency` column in the `campaign_performance` table represents the average number of times a user was exposed to an ad. It is a directly recorded metric within the table, not a derived field from other columns in this schema.</t>
+          <t>The database schema does not contain information on how the `frequency` column in the `campaign_performance` table is derived. It only indicates that it is a FLOAT type.</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.836</v>
+        <v>0.789</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[{'invocationId': 'e-83203d58-7476-40f2-aa64-646157beb36e', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'yNynCm25', 'timestamp': 1757072566.122553}, {'content': {'parts': [{'text': 'The `frequency` column in the `campaign_performance` table represents the average number of times a user was exposed to an ad. It is a directly recorded metric within the table, not a derived field from other columns in this schema.'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 48, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 48}], 'promptTokenCount': 8238, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8238}], 'thoughtsTokenCount': 87, 'totalTokenCount': 8373, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-83203d58-7476-40f2-aa64-646157beb36e', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'Lq2HFlnm', 'timestamp': 1757072566.124085}]</t>
+          <t>[{'invocationId': 'e-afb7e838-5559-47f2-9705-84ffc1621fe4', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': '3HkvMpmW', 'timestamp': 1757408396.074303}, {'content': {'parts': [{'text': 'The database schema does not contain information on how the `frequency` column in the `campaign_performance` table is derived. It only indicates that it is a FLOAT type.'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 35, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 35}], 'promptTokenCount': 8238, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8238}], 'thoughtsTokenCount': 145, 'totalTokenCount': 8418, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-afb7e838-5559-47f2-9705-84ffc1621fe4', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'FKZBL9e1', 'timestamp': 1757408396.079495}]</t>
         </is>
       </c>
     </row>
@@ -512,12 +512,11 @@
 *   `campaign_id`
 *   `campaign_ad_id`
 *   `brand_id`
-*   `brand_name`
-*   `product_ids` (Note: `transaction_data` has `sku_id` which is a product identifier, and `campaign_performance` has `product_ids`. These are likely related and can be used for linking, but `campaign_id`, `campaign_ad_id`, `brand_id`, and `brand_name` are direct common fields.)</t>
+*   `brand_name`</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.806</v>
+        <v>0.889</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -526,7 +525,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[{'invocationId': 'e-53e9ea95-dcb7-49ea-9e32-cb36aa084b26', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': '76tvzSiR', 'timestamp': 1757072575.663537}, {'content': {'parts': [{'text': 'The `transaction_data` and `campaign_performance` tables can be linked using the following fields:\n\n*   `campaign_id`\n*   `campaign_ad_id`\n*   `brand_id`\n*   `brand_name`\n*   `product_ids` (Note: `transaction_data` has `sku_id` which is a product identifier, and `campaign_performance` has `product_ids`. These are likely related and can be used for linking, but `campaign_id`, `campaign_ad_id`, `brand_id`, and `brand_name` are direct common fields.)'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 135, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 135}], 'promptTokenCount': 8241, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8241}], 'thoughtsTokenCount': 359, 'totalTokenCount': 8735, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-53e9ea95-dcb7-49ea-9e32-cb36aa084b26', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'UyxqDIA6', 'timestamp': 1757072575.665663}]</t>
+          <t>[{'invocationId': 'e-345329c7-dffb-49e8-a273-fa9b3f780d03', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'LGTAye05', 'timestamp': 1757408405.638018}, {'content': {'parts': [{'text': 'The `transaction_data` and `campaign_performance` tables can be linked using the following fields:\n\n*   `campaign_id`\n*   `campaign_ad_id`\n*   `brand_id`\n*   `brand_name`'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 55, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 55}], 'promptTokenCount': 8241, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8241}], 'thoughtsTokenCount': 514, 'totalTokenCount': 8810, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-345329c7-dffb-49e8-a273-fa9b3f780d03', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'CBMk6ekb', 'timestamp': 1757408405.644448}]</t>
         </is>
       </c>
     </row>
@@ -544,20 +543,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CPC is a direct column in the `campaign_performance` table.</t>
+          <t>Result: CPC (Cost Per Click) in the `campaign_performance` table is calculated as `actual_spend_to_date / clicks`. This means it's the total amount spent on the campaign divided by the total number of clicks received.</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.733</v>
+        <v>0.931</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[{'invocationId': 'e-38fb7be2-f610-4fad-a483-2cfd54bb351c', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'xsODIdc6', 'timestamp': 1757072586.172655}, {'content': {'parts': [{'text': 'CPC is a direct column in the `campaign_performance` table.'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7609}], 'cachedContentTokenCount': 7609, 'candidatesTokenCount': 14, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 14}], 'promptTokenCount': 8237, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8237}], 'thoughtsTokenCount': 206, 'totalTokenCount': 8457, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-38fb7be2-f610-4fad-a483-2cfd54bb351c', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'kzpeQkDN', 'timestamp': 1757072586.175194}]</t>
+          <t>[{'invocationId': 'e-55acbcac-2475-402d-a87b-1c0e2c31fcb0', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'B7blYugO', 'timestamp': 1757408416.643002}, {'content': {'parts': [{'functionCall': {'id': 'adk-eecbb920-9953-4610-b436-4298336ff580', 'args': {'question': 'How is CPC calculated in the campaign_performance table?'}, 'name': 'call_db_agent'}}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7609}], 'cachedContentTokenCount': 7609, 'candidatesTokenCount': 17, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 17}], 'promptTokenCount': 8237, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8237}], 'thoughtsTokenCount': 134, 'totalTokenCount': 8388, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-55acbcac-2475-402d-a87b-1c0e2c31fcb0', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'longRunningToolIds': [], 'id': 'r042ffmV', 'timestamp': 1757408416.646525}, {'content': {'parts': [{'functionResponse': {'id': 'adk-eecbb920-9953-4610-b436-4298336ff580', 'name': 'call_db_agent', 'response': {'result': "CPC (Cost Per Click) in the `campaign_performance` table is calculated as `actual_spend_to_date / clicks`. This means it's the total amount spent on the campaign divided by the total number of clicks received."}}}], 'role': 'user'}, 'invocationId': 'e-55acbcac-2475-402d-a87b-1c0e2c31fcb0', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'db_agent_output': "CPC (Cost Per Click) in the `campaign_performance` table is calculated as `actual_spend_to_date / clicks`. This means it's the total amount spent on the campaign divided by the total number of clicks received."}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'OjZqJ2Vg', 'timestamp': 1757408435.521191}, {'content': {'parts': [{'text': "Result: CPC (Cost Per Click) in the `campaign_performance` table is calculated as `actual_spend_to_date / clicks`. This means it's the total amount spent on the campaign divided by the total number of clicks received."}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7587}], 'cachedContentTokenCount': 7587, 'candidatesTokenCount': 51, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 51}], 'promptTokenCount': 8309, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8309}], 'thoughtsTokenCount': 88, 'totalTokenCount': 8448, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-55acbcac-2475-402d-a87b-1c0e2c31fcb0', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'JgCK2n4k', 'timestamp': 1757408435.521191}]</t>
         </is>
       </c>
     </row>
@@ -576,11 +575,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>`conversion_rate_percent` in the `campaign_performance` table is defined as a `FLOAT`.</t>
+          <t>`conversion_rate_percent` in the `campaign_performance` table is defined as a FLOAT. It represents the conversion rate in percentage.</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.883</v>
+        <v>0.926</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -589,7 +588,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[{'invocationId': 'e-33020a5b-8ce4-4a63-af12-c09802a704a8', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'nYnykQcL', 'timestamp': 1757072596.815562}, {'content': {'parts': [{'text': '`conversion_rate_percent` in the `campaign_performance` table is defined as a `FLOAT`.'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 22, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 22}], 'promptTokenCount': 8242, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8242}], 'thoughtsTokenCount': 117, 'totalTokenCount': 8381, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-33020a5b-8ce4-4a63-af12-c09802a704a8', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'vrCwuBmT', 'timestamp': 1757072596.816599}]</t>
+          <t>[{'invocationId': 'e-daddcbe7-3cfb-4228-b8d9-028dcdcf41bb', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {'all_db_settings': {'use_database': 'BigQuery'}, 'database_settings': {'bq_project_id': 'acn-cda', 'bq_dataset_id': 'RMN_Campaign_Dataset_Dev', 'bq_ddl_schema': "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','≥ 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", 'transpile_to_bigquery': True, 'process_input_errors': True, 'process_tool_output_errors': True, 'number_of_candidates': 1, 'model': 'gemini-2.5-flash', 'temperature': 0.01, 'generate_sql_type': 'dc'}}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'dIXI7nsD', 'timestamp': 1757408444.218784}, {'content': {'parts': [{'text': '`conversion_rate_percent` in the `campaign_performance` table is defined as a FLOAT. It represents the conversion rate in percentage.'}], 'role': 'model'}, 'usageMetadata': {'cacheTokensDetails': [{'modality': 'TEXT', 'tokenCount': 7610}], 'cachedContentTokenCount': 7610, 'candidatesTokenCount': 29, 'candidatesTokensDetails': [{'modality': 'TEXT', 'tokenCount': 29}], 'promptTokenCount': 8242, 'promptTokensDetails': [{'modality': 'TEXT', 'tokenCount': 8242}], 'thoughtsTokenCount': 142, 'totalTokenCount': 8413, 'trafficType': 'ON_DEMAND'}, 'invocationId': 'e-daddcbe7-3cfb-4228-b8d9-028dcdcf41bb', 'author': 'db_ds_multiagent', 'actions': {'stateDelta': {}, 'artifactDelta': {}, 'requestedAuthConfigs': {}}, 'id': 'FOROC2rO', 'timestamp': 1757408444.23063}]</t>
         </is>
       </c>
     </row>

</xml_diff>